<commit_message>
New file path for new computer
</commit_message>
<xml_diff>
--- a/top_250_data.xlsx
+++ b/top_250_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C269"/>
+  <dimension ref="A1:C282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4456,14 +4456,217 @@
           <t>Streetwise</t>
         </is>
       </c>
-      <c r="B269" t="inlineStr">
-        <is>
-          <t>1984</t>
-        </is>
+      <c r="B269" t="n">
+        <v>1984</v>
       </c>
       <c r="C269" t="inlineStr">
         <is>
           <t>https://letterboxd.com/film/streetwise/</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Taylor Swift | The Eras Tour | The Final Show</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/taylor-swift-the-eras-tour-the-final-show/</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>The End of an Era</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/the-end-of-an-era-2025/</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Sufjan Stevens: Carrie &amp; Lowell Live</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/sufjan-stevens-carrie-lowell-live-2017/</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Cabaret</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>1993</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/cabaret-1993/</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Michael Jackson's Thriller</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>1983</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/michael-jacksons-thriller/</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Farewell My Concubine</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>1993</v>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/farewell-my-concubine/</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Cosmos</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>2014</v>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/cosmos-2014/</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>j-hope Tour 'HOPE ON THE STAGE' in JAPAN: LIVE VIEWING</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/j-hope-tour-hope-on-the-stage-in-japan-live/</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>No me quiero ir de aquí: Una más</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/no-me-quiero-ir-de-aqui-una-mas-2025/</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Fiona Apple: MTV Live in New York, 1999</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>1999</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/fiona-apple-mtv-live-in-new-york-1999/</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>The Voice of Hind Rajab</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/the-voice-of-hind-rajab/</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Attack on Titan: Crimson Bow and Arrow</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/attack-on-titan-crimson-bow-and-arrow/</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Twenty One Pilots: MTV Unplugged</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/twenty-one-pilots-mtv-unplugged/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Updating to use Chrome
</commit_message>
<xml_diff>
--- a/top_250_data.xlsx
+++ b/top_250_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C284"/>
+  <dimension ref="A1:C285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4666,10 +4666,8 @@
           <t>Twenty One Pilots: More Than We Ever Imagined</t>
         </is>
       </c>
-      <c r="B283" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
+      <c r="B283" t="n">
+        <v>2026</v>
       </c>
       <c r="C283" t="inlineStr">
         <is>
@@ -4683,14 +4681,29 @@
           <t>Red Hot Chili Peppers: Live at Slane Castle</t>
         </is>
       </c>
-      <c r="B284" t="inlineStr">
-        <is>
-          <t>2003</t>
-        </is>
+      <c r="B284" t="n">
+        <v>2003</v>
       </c>
       <c r="C284" t="inlineStr">
         <is>
           <t>https://letterboxd.com/film/red-hot-chili-peppers-live-at-slane-castle-2003/</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>The Phantom of the Opera at the Royal Albert Hall</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/the-phantom-of-the-opera-at-the-royal-albert-hall/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adding batching. Fixing bug.
</commit_message>
<xml_diff>
--- a/top_250_data.xlsx
+++ b/top_250_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D304"/>
+  <dimension ref="A1:D305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6064,10 +6064,8 @@
           <t>Sassy the Sasquatch</t>
         </is>
       </c>
-      <c r="B303" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
+      <c r="B303" t="n">
+        <v>2022</v>
       </c>
       <c r="C303" t="inlineStr">
         <is>
@@ -6082,10 +6080,8 @@
           <t>HOMECOMING: A film by Beyoncé</t>
         </is>
       </c>
-      <c r="B304" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
+      <c r="B304" t="n">
+        <v>2019</v>
       </c>
       <c r="C304" t="inlineStr">
         <is>
@@ -6095,6 +6091,28 @@
       <c r="D304" t="inlineStr">
         <is>
           <t>593691</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Interview with the Vampire</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/interview-with-the-vampire-2022/</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>921618</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adding official/regular list distinctions
</commit_message>
<xml_diff>
--- a/top_250_data.xlsx
+++ b/top_250_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D311"/>
+  <dimension ref="A1:D313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6180,10 +6180,8 @@
           <t>Banana Fish</t>
         </is>
       </c>
-      <c r="B309" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
+      <c r="B309" t="n">
+        <v>2018</v>
       </c>
       <c r="C309" t="inlineStr">
         <is>
@@ -6198,10 +6196,8 @@
           <t>Ticket to Heaven</t>
         </is>
       </c>
-      <c r="B310" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
+      <c r="B310" t="n">
+        <v>2026</v>
       </c>
       <c r="C310" t="inlineStr">
         <is>
@@ -6216,10 +6212,8 @@
           <t>Swing Girls</t>
         </is>
       </c>
-      <c r="B311" t="inlineStr">
-        <is>
-          <t>2004</t>
-        </is>
+      <c r="B311" t="n">
+        <v>2004</v>
       </c>
       <c r="C311" t="inlineStr">
         <is>
@@ -6229,6 +6223,50 @@
       <c r="D311" t="inlineStr">
         <is>
           <t>36592</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Gravity Falls: Between the Pines</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/gravity-falls-between-the-pines/</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>1602449</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>SUGA | Agust D TOUR 'D-DAY' THE MOVIE</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>https://letterboxd.com/film/suga-agust-d-tour-d-day-the-movie/</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>1254724</t>
         </is>
       </c>
     </row>

</xml_diff>